<commit_message>
feat: process new records from LetterLog.xlsx
</commit_message>
<xml_diff>
--- a/LetterLog.xlsx
+++ b/LetterLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Muhammad Ali Qamar\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD368A53-745D-4A7D-A7D6-96751E03C764}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{941141D8-85F3-496E-9C17-59F0600CAECF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="20">
   <si>
     <t>Reference Number</t>
   </si>
@@ -63,29 +63,35 @@
     <t>Annexure I – Terms and Conditions</t>
   </si>
   <si>
-    <t>DL-HRM-INT-26-0239</t>
-  </si>
-  <si>
-    <t>DL-HRM-INT-26-0240</t>
-  </si>
-  <si>
-    <t>DL-HRM-INT-26-0241</t>
-  </si>
-  <si>
-    <t>Rida Naseer</t>
-  </si>
-  <si>
-    <t>Sarah Khan</t>
-  </si>
-  <si>
-    <t>Amna Arshad Butt</t>
+    <t>DL-HRM-INT-26-0242</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0243</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0244</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0245</t>
+  </si>
+  <si>
+    <t>Hashim Matloob Raja</t>
+  </si>
+  <si>
+    <t>Alishba Amin Joyia</t>
+  </si>
+  <si>
+    <t>Abdullah Bin Masood</t>
+  </si>
+  <si>
+    <t>Sawaiz Tanveer</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -105,6 +111,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -127,11 +139,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -471,7 +484,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
@@ -510,8 +523,8 @@
       <c r="A2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" t="s">
-        <v>15</v>
+      <c r="B2" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="C2" t="s">
         <v>9</v>
@@ -534,7 +547,7 @@
         <v>13</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
         <v>9</v>
@@ -557,7 +570,7 @@
         <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
         <v>9</v>
@@ -572,6 +585,29 @@
         <v>10</v>
       </c>
       <c r="G4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5" t="s">
         <v>11</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: ingest 35 records from LetterLog.xlsx and generate bulk QR codes
</commit_message>
<xml_diff>
--- a/LetterLog.xlsx
+++ b/LetterLog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Muhammad Ali Qamar\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{941141D8-85F3-496E-9C17-59F0600CAECF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D943844E-7325-43D9-9F24-50BB61D0C8C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="82">
   <si>
     <t>Reference Number</t>
   </si>
@@ -54,37 +54,223 @@
     <t>Chief Executive Officer</t>
   </si>
   <si>
-    <t>24th July, 2026</t>
-  </si>
-  <si>
     <t>Internship Offer Letter</t>
   </si>
   <si>
     <t>Annexure I – Terms and Conditions</t>
   </si>
   <si>
-    <t>DL-HRM-INT-26-0242</t>
-  </si>
-  <si>
-    <t>DL-HRM-INT-26-0243</t>
-  </si>
-  <si>
-    <t>DL-HRM-INT-26-0244</t>
-  </si>
-  <si>
-    <t>DL-HRM-INT-26-0245</t>
-  </si>
-  <si>
-    <t>Hashim Matloob Raja</t>
-  </si>
-  <si>
-    <t>Alishba Amin Joyia</t>
-  </si>
-  <si>
-    <t>Abdullah Bin Masood</t>
-  </si>
-  <si>
-    <t>Sawaiz Tanveer</t>
+    <t>DL-HRM-INT-26-0246</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0247</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0248</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0249</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0250</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0251</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0252</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0253</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0254</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0255</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0256</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0257</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0258</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0259</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0260</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0261</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0262</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0263</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0264</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0265</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0266</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0267</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0268</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0269</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0270</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0271</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0272</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0273</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0274</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0275</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0276</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0277</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0278</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0279</t>
+  </si>
+  <si>
+    <t>DL-HRM-INT-26-0280</t>
+  </si>
+  <si>
+    <t>25th July, 2026</t>
+  </si>
+  <si>
+    <t>Muhammad Zohaib Raza</t>
+  </si>
+  <si>
+    <t>Umaima Shahid</t>
+  </si>
+  <si>
+    <t>Muhammad Haris</t>
+  </si>
+  <si>
+    <t>Muhammad Fahad Hussain</t>
+  </si>
+  <si>
+    <t>Anila Younas</t>
+  </si>
+  <si>
+    <t>Faiza Marrium</t>
+  </si>
+  <si>
+    <t>Zain Jamshaid</t>
+  </si>
+  <si>
+    <t>Haleema Jawad</t>
+  </si>
+  <si>
+    <t>Hamna Waqar</t>
+  </si>
+  <si>
+    <t>Hamna Hameed</t>
+  </si>
+  <si>
+    <t>Kisa Batool</t>
+  </si>
+  <si>
+    <t>Noor Fatima</t>
+  </si>
+  <si>
+    <t>Fatima Nadeem</t>
+  </si>
+  <si>
+    <t>Hadiqa Tul Eman Kashmira</t>
+  </si>
+  <si>
+    <t>Laiba Noor</t>
+  </si>
+  <si>
+    <t>Zainab Batool</t>
+  </si>
+  <si>
+    <t>Areesha Sarwar</t>
+  </si>
+  <si>
+    <t>Minahil Imran</t>
+  </si>
+  <si>
+    <t>Sayyda Arooj</t>
+  </si>
+  <si>
+    <t>Fatima Ijaz</t>
+  </si>
+  <si>
+    <t>Mahrukh Zeshan</t>
+  </si>
+  <si>
+    <t>Kaneez Fatima</t>
+  </si>
+  <si>
+    <t>Atiqa Maqbool</t>
+  </si>
+  <si>
+    <t>Aqsa Noor</t>
+  </si>
+  <si>
+    <t>Muhammad Fareed</t>
+  </si>
+  <si>
+    <t>Muhammad Mubeen Khan</t>
+  </si>
+  <si>
+    <t>Muhammad Omair Akbar</t>
+  </si>
+  <si>
+    <t>ibrahim</t>
+  </si>
+  <si>
+    <t>Suliman Badar Butt</t>
+  </si>
+  <si>
+    <t>Ahtisham Mohsin</t>
+  </si>
+  <si>
+    <t>Sanjai</t>
+  </si>
+  <si>
+    <t>Halima Sadia</t>
+  </si>
+  <si>
+    <t>Muskan</t>
+  </si>
+  <si>
+    <t>Momna</t>
+  </si>
+  <si>
+    <t>Momna Hafeez</t>
   </si>
 </sst>
 </file>
@@ -484,11 +670,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
+    <col min="2" max="2" width="23.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.83203125" customWidth="1"/>
     <col min="4" max="4" width="22.83203125" customWidth="1"/>
     <col min="5" max="5" width="25.83203125" customWidth="1"/>
@@ -521,13 +707,13 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>16</v>
+        <v>71</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>46</v>
       </c>
       <c r="D2" t="s">
         <v>7</v>
@@ -536,21 +722,21 @@
         <v>8</v>
       </c>
       <c r="F2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>46</v>
       </c>
       <c r="D3" t="s">
         <v>7</v>
@@ -559,21 +745,21 @@
         <v>8</v>
       </c>
       <c r="F3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
+        <v>46</v>
       </c>
       <c r="D4" t="s">
         <v>7</v>
@@ -582,40 +768,753 @@
         <v>8</v>
       </c>
       <c r="F4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
         <v>15</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" t="s">
+        <v>50</v>
+      </c>
+      <c r="C7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" t="s">
+        <v>73</v>
+      </c>
+      <c r="C8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F8" t="s">
+        <v>9</v>
+      </c>
+      <c r="G8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C9" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" t="s">
+        <v>8</v>
+      </c>
+      <c r="F9" t="s">
+        <v>9</v>
+      </c>
+      <c r="G9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>19</v>
       </c>
-      <c r="C5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" t="s">
-        <v>10</v>
-      </c>
-      <c r="G5" t="s">
-        <v>11</v>
+      <c r="B10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+      <c r="G10" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" t="s">
+        <v>75</v>
+      </c>
+      <c r="C11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" t="s">
+        <v>8</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+      <c r="G11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C12" t="s">
+        <v>46</v>
+      </c>
+      <c r="D12" t="s">
+        <v>7</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+      <c r="G12" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C13" t="s">
+        <v>46</v>
+      </c>
+      <c r="D13" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" t="s">
+        <v>9</v>
+      </c>
+      <c r="G13" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F14" t="s">
+        <v>9</v>
+      </c>
+      <c r="G14" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" t="s">
+        <v>54</v>
+      </c>
+      <c r="C15" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" t="s">
+        <v>9</v>
+      </c>
+      <c r="G15" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" t="s">
+        <v>55</v>
+      </c>
+      <c r="C16" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="F16" t="s">
+        <v>9</v>
+      </c>
+      <c r="G16" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" t="s">
+        <v>56</v>
+      </c>
+      <c r="C17" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" t="s">
+        <v>7</v>
+      </c>
+      <c r="E17" t="s">
+        <v>8</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+      <c r="G17" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" t="s">
+        <v>46</v>
+      </c>
+      <c r="D18" t="s">
+        <v>7</v>
+      </c>
+      <c r="E18" t="s">
+        <v>8</v>
+      </c>
+      <c r="F18" t="s">
+        <v>9</v>
+      </c>
+      <c r="G18" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>28</v>
+      </c>
+      <c r="B19" t="s">
+        <v>77</v>
+      </c>
+      <c r="C19" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" t="s">
+        <v>7</v>
+      </c>
+      <c r="E19" t="s">
+        <v>8</v>
+      </c>
+      <c r="F19" t="s">
+        <v>9</v>
+      </c>
+      <c r="G19" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>29</v>
+      </c>
+      <c r="B20" t="s">
+        <v>58</v>
+      </c>
+      <c r="C20" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" t="s">
+        <v>7</v>
+      </c>
+      <c r="E20" t="s">
+        <v>8</v>
+      </c>
+      <c r="F20" t="s">
+        <v>9</v>
+      </c>
+      <c r="G20" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>30</v>
+      </c>
+      <c r="B21" t="s">
+        <v>59</v>
+      </c>
+      <c r="C21" t="s">
+        <v>46</v>
+      </c>
+      <c r="D21" t="s">
+        <v>7</v>
+      </c>
+      <c r="E21" t="s">
+        <v>8</v>
+      </c>
+      <c r="F21" t="s">
+        <v>9</v>
+      </c>
+      <c r="G21" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>31</v>
+      </c>
+      <c r="B22" t="s">
+        <v>60</v>
+      </c>
+      <c r="C22" t="s">
+        <v>46</v>
+      </c>
+      <c r="D22" t="s">
+        <v>7</v>
+      </c>
+      <c r="E22" t="s">
+        <v>8</v>
+      </c>
+      <c r="F22" t="s">
+        <v>9</v>
+      </c>
+      <c r="G22" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23" t="s">
+        <v>61</v>
+      </c>
+      <c r="C23" t="s">
+        <v>46</v>
+      </c>
+      <c r="D23" t="s">
+        <v>7</v>
+      </c>
+      <c r="E23" t="s">
+        <v>8</v>
+      </c>
+      <c r="F23" t="s">
+        <v>9</v>
+      </c>
+      <c r="G23" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>33</v>
+      </c>
+      <c r="B24" t="s">
+        <v>78</v>
+      </c>
+      <c r="C24" t="s">
+        <v>46</v>
+      </c>
+      <c r="D24" t="s">
+        <v>7</v>
+      </c>
+      <c r="E24" t="s">
+        <v>8</v>
+      </c>
+      <c r="F24" t="s">
+        <v>9</v>
+      </c>
+      <c r="G24" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>34</v>
+      </c>
+      <c r="B25" t="s">
+        <v>79</v>
+      </c>
+      <c r="C25" t="s">
+        <v>46</v>
+      </c>
+      <c r="D25" t="s">
+        <v>7</v>
+      </c>
+      <c r="E25" t="s">
+        <v>8</v>
+      </c>
+      <c r="F25" t="s">
+        <v>9</v>
+      </c>
+      <c r="G25" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>35</v>
+      </c>
+      <c r="B26" t="s">
+        <v>80</v>
+      </c>
+      <c r="C26" t="s">
+        <v>46</v>
+      </c>
+      <c r="D26" t="s">
+        <v>7</v>
+      </c>
+      <c r="E26" t="s">
+        <v>8</v>
+      </c>
+      <c r="F26" t="s">
+        <v>9</v>
+      </c>
+      <c r="G26" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>36</v>
+      </c>
+      <c r="B27" t="s">
+        <v>62</v>
+      </c>
+      <c r="C27" t="s">
+        <v>46</v>
+      </c>
+      <c r="D27" t="s">
+        <v>7</v>
+      </c>
+      <c r="E27" t="s">
+        <v>8</v>
+      </c>
+      <c r="F27" t="s">
+        <v>9</v>
+      </c>
+      <c r="G27" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>37</v>
+      </c>
+      <c r="B28" t="s">
+        <v>63</v>
+      </c>
+      <c r="C28" t="s">
+        <v>46</v>
+      </c>
+      <c r="D28" t="s">
+        <v>7</v>
+      </c>
+      <c r="E28" t="s">
+        <v>8</v>
+      </c>
+      <c r="F28" t="s">
+        <v>9</v>
+      </c>
+      <c r="G28" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>38</v>
+      </c>
+      <c r="B29" t="s">
+        <v>64</v>
+      </c>
+      <c r="C29" t="s">
+        <v>46</v>
+      </c>
+      <c r="D29" t="s">
+        <v>7</v>
+      </c>
+      <c r="E29" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" t="s">
+        <v>9</v>
+      </c>
+      <c r="G29" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>39</v>
+      </c>
+      <c r="B30" t="s">
+        <v>65</v>
+      </c>
+      <c r="C30" t="s">
+        <v>46</v>
+      </c>
+      <c r="D30" t="s">
+        <v>7</v>
+      </c>
+      <c r="E30" t="s">
+        <v>8</v>
+      </c>
+      <c r="F30" t="s">
+        <v>9</v>
+      </c>
+      <c r="G30" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>40</v>
+      </c>
+      <c r="B31" t="s">
+        <v>81</v>
+      </c>
+      <c r="C31" t="s">
+        <v>46</v>
+      </c>
+      <c r="D31" t="s">
+        <v>7</v>
+      </c>
+      <c r="E31" t="s">
+        <v>8</v>
+      </c>
+      <c r="F31" t="s">
+        <v>9</v>
+      </c>
+      <c r="G31" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>41</v>
+      </c>
+      <c r="B32" t="s">
+        <v>66</v>
+      </c>
+      <c r="C32" t="s">
+        <v>46</v>
+      </c>
+      <c r="D32" t="s">
+        <v>7</v>
+      </c>
+      <c r="E32" t="s">
+        <v>8</v>
+      </c>
+      <c r="F32" t="s">
+        <v>9</v>
+      </c>
+      <c r="G32" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>42</v>
+      </c>
+      <c r="B33" t="s">
+        <v>67</v>
+      </c>
+      <c r="C33" t="s">
+        <v>46</v>
+      </c>
+      <c r="D33" t="s">
+        <v>7</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
+      <c r="F33" t="s">
+        <v>9</v>
+      </c>
+      <c r="G33" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>43</v>
+      </c>
+      <c r="B34" t="s">
+        <v>68</v>
+      </c>
+      <c r="C34" t="s">
+        <v>46</v>
+      </c>
+      <c r="D34" t="s">
+        <v>7</v>
+      </c>
+      <c r="E34" t="s">
+        <v>8</v>
+      </c>
+      <c r="F34" t="s">
+        <v>9</v>
+      </c>
+      <c r="G34" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>44</v>
+      </c>
+      <c r="B35" t="s">
+        <v>69</v>
+      </c>
+      <c r="C35" t="s">
+        <v>46</v>
+      </c>
+      <c r="D35" t="s">
+        <v>7</v>
+      </c>
+      <c r="E35" t="s">
+        <v>8</v>
+      </c>
+      <c r="F35" t="s">
+        <v>9</v>
+      </c>
+      <c r="G35" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>45</v>
+      </c>
+      <c r="B36" t="s">
+        <v>70</v>
+      </c>
+      <c r="C36" t="s">
+        <v>46</v>
+      </c>
+      <c r="D36" t="s">
+        <v>7</v>
+      </c>
+      <c r="E36" t="s">
+        <v>8</v>
+      </c>
+      <c r="F36" t="s">
+        <v>9</v>
+      </c>
+      <c r="G36" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:G1 C2:E2" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:G1 D2:E2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>